<commit_message>
Add Youtube videos to TP and WTS
</commit_message>
<xml_diff>
--- a/pages/video_analysis/WTS_Master_Women.xlsx
+++ b/pages/video_analysis/WTS_Master_Women.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sportnzgroup-my.sharepoint.com/personal/anja_kuys_hpsnz_org_nz/Documents/Desktop/Scripts/CNZPD/pages/video_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{262EE144-5106-46E3-9413-1E8BB520A031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8D09A51-849D-4BFF-9B72-4E1564EF6BF8}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{262EE144-5106-46E3-9413-1E8BB520A031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25C280FD-541B-4B2E-AE68-ACCF94820EC0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1620" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5737" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5738" uniqueCount="223">
   <si>
     <t>Title</t>
   </si>
@@ -687,6 +687,9 @@
   <si>
     <t>26-07-30 CWG Glasgow NZL Q</t>
   </si>
+  <si>
+    <t>https://youtu.be/-DxHcKVATsM</t>
+  </si>
 </sst>
 </file>
 
@@ -44577,7 +44580,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2513" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2513" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2513" t="s">
         <v>220</v>
       </c>
@@ -44594,7 +44597,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2514" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2514" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2514" t="s">
         <v>220</v>
       </c>
@@ -44611,7 +44614,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2515" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2515" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2515" t="s">
         <v>220</v>
       </c>
@@ -44628,7 +44631,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2516" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2516" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2516" t="s">
         <v>220</v>
       </c>
@@ -44645,7 +44648,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2517" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2517" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2517" t="s">
         <v>220</v>
       </c>
@@ -44662,7 +44665,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2518" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2518" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2518" t="s">
         <v>220</v>
       </c>
@@ -44679,7 +44682,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2519" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2519" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2519" t="s">
         <v>220</v>
       </c>
@@ -44696,7 +44699,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2520" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2520" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2520" t="s">
         <v>220</v>
       </c>
@@ -44713,7 +44716,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2521" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2521" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2521" t="s">
         <v>220</v>
       </c>
@@ -44730,7 +44733,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2522" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2522" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2522" t="s">
         <v>221</v>
       </c>
@@ -44743,8 +44746,11 @@
       <c r="D2522" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="2523" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="G2522" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2523" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2523" t="s">
         <v>221</v>
       </c>
@@ -44758,7 +44764,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="2524" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2524" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2524" t="s">
         <v>221</v>
       </c>
@@ -44772,7 +44778,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="2525" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2525" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2525" t="s">
         <v>221</v>
       </c>
@@ -44783,7 +44789,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2526" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2526" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2526" t="s">
         <v>221</v>
       </c>
@@ -44794,7 +44800,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2527" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2527" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2527" t="s">
         <v>221</v>
       </c>
@@ -44805,7 +44811,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2528" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2528" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2528" t="s">
         <v>221</v>
       </c>

</xml_diff>